<commit_message>
Archive FY26 files and update current versions
Archive previous FY26 versions of Preassignments, Preferences, Requirements, and Tracks to FY26 Archive folder. Update the working copies in upload files directory with new versions.
</commit_message>
<xml_diff>
--- a/upload files/Preassignments.xlsx
+++ b/upload files/Preassignments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29022"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\MedFlight Docs\Rebid Shift Tool\5.20.25\5-21-25\upload files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aaronbell/Desktop/Git Repo Clone/CrewOps360/upload files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{838FC3A7-D5D2-4630-B3AE-1875C2670C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC96E6D9-656C-4C65-831B-B149C3AF39B2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE0FF30-FAB5-A44C-B396-DF2AAD78374A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30330" yWindow="1560" windowWidth="27270" windowHeight="14520" xr2:uid="{011E8F27-AA14-4802-A81C-8523FD4162A1}"/>
+    <workbookView xWindow="1100" yWindow="1040" windowWidth="27280" windowHeight="14520" xr2:uid="{011E8F27-AA14-4802-A81C-8523FD4162A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="55">
   <si>
     <t>STAFF NAME</t>
   </si>
@@ -182,9 +182,6 @@
     <t>Hanley-McCarthy</t>
   </si>
   <si>
-    <t>Hourihan</t>
-  </si>
-  <si>
     <t>Mee</t>
   </si>
   <si>
@@ -195,13 +192,22 @@
   </si>
   <si>
     <t>Rabickow</t>
+  </si>
+  <si>
+    <t>Timm</t>
+  </si>
+  <si>
+    <t>Montano</t>
+  </si>
+  <si>
+    <t>Laterion</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,7 +322,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -343,6 +349,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -679,56 +688,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F22AD928-7495-4B5C-89C3-15EF76B28594}">
-  <dimension ref="A1:AQ10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:AQ12"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.5" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.5" style="4" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.5" style="4" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="7.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="7.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="4"/>
+    <col min="25" max="25" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="6.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="7.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="44" max="16384" width="9.1640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="15.75" thickBot="1">
+    <row r="1" spans="1:43" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -859,254 +868,615 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:43">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="B2" s="5"/>
-      <c r="J2" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
       <c r="O2" s="6"/>
       <c r="P2" s="5"/>
-      <c r="Q2" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q2" s="10"/>
+      <c r="R2" s="10"/>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+      <c r="V2" s="10"/>
+      <c r="W2" s="10"/>
+      <c r="X2" s="10"/>
+      <c r="Y2" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z2" s="10"/>
+      <c r="AA2" s="10"/>
+      <c r="AB2" s="10"/>
       <c r="AC2" s="6"/>
       <c r="AD2" s="5"/>
-      <c r="AL2" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE2" s="10"/>
+      <c r="AF2" s="10"/>
+      <c r="AG2" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH2" s="10"/>
+      <c r="AI2" s="10"/>
+      <c r="AJ2" s="10"/>
+      <c r="AK2" s="10"/>
+      <c r="AL2" s="10"/>
+      <c r="AM2" s="10"/>
+      <c r="AN2" s="10"/>
+      <c r="AO2" s="10"/>
+      <c r="AP2" s="10"/>
       <c r="AQ2" s="6"/>
     </row>
-    <row r="3" spans="1:43">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B3" s="5"/>
-      <c r="E3" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
+      <c r="L3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="M3" s="10"/>
+      <c r="N3" s="10"/>
       <c r="O3" s="6"/>
       <c r="P3" s="5"/>
-      <c r="S3" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="10"/>
+      <c r="S3" s="10"/>
+      <c r="T3" s="10"/>
+      <c r="U3" s="10"/>
+      <c r="V3" s="10"/>
+      <c r="W3" s="10"/>
+      <c r="X3" s="10"/>
+      <c r="Y3" s="10"/>
+      <c r="Z3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA3" s="10"/>
+      <c r="AB3" s="10"/>
       <c r="AC3" s="6"/>
       <c r="AD3" s="5"/>
-      <c r="AG3" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE3" s="10"/>
+      <c r="AF3" s="10"/>
+      <c r="AG3" s="10"/>
+      <c r="AH3" s="10"/>
+      <c r="AI3" s="10"/>
+      <c r="AJ3" s="10"/>
+      <c r="AK3" s="10"/>
+      <c r="AL3" s="10"/>
+      <c r="AM3" s="10"/>
+      <c r="AN3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO3" s="10"/>
+      <c r="AP3" s="10"/>
       <c r="AQ3" s="6"/>
     </row>
-    <row r="4" spans="1:43">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B4" s="5"/>
-      <c r="E4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" s="10"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
       <c r="O4" s="6"/>
       <c r="P4" s="5"/>
-      <c r="S4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA4" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S4" s="10"/>
+      <c r="T4" s="10"/>
+      <c r="U4" s="10"/>
+      <c r="V4" s="10"/>
+      <c r="W4" s="10"/>
+      <c r="X4" s="10"/>
+      <c r="Y4" s="10"/>
+      <c r="Z4" s="10"/>
+      <c r="AA4" s="10"/>
+      <c r="AB4" s="10"/>
       <c r="AC4" s="6"/>
       <c r="AD4" s="5"/>
-      <c r="AH4" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="AN4" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE4" s="10"/>
+      <c r="AF4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG4" s="10"/>
+      <c r="AH4" s="10"/>
+      <c r="AI4" s="10"/>
+      <c r="AJ4" s="10"/>
+      <c r="AK4" s="10"/>
+      <c r="AL4" s="10"/>
+      <c r="AM4" s="10"/>
+      <c r="AN4" s="10"/>
+      <c r="AO4" s="10"/>
+      <c r="AP4" s="10"/>
       <c r="AQ4" s="6"/>
     </row>
-    <row r="5" spans="1:43">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B5" s="5"/>
-      <c r="C5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="10"/>
+      <c r="F5" s="10"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
       <c r="O5" s="6"/>
       <c r="P5" s="5"/>
-      <c r="R5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="X5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y5" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="R5" s="10"/>
+      <c r="S5" s="10"/>
+      <c r="T5" s="10"/>
+      <c r="U5" s="10"/>
+      <c r="V5" s="10"/>
+      <c r="W5" s="10"/>
+      <c r="X5" s="10"/>
+      <c r="Y5" s="10"/>
+      <c r="Z5" s="10"/>
+      <c r="AA5" s="10"/>
+      <c r="AB5" s="10"/>
       <c r="AC5" s="6"/>
       <c r="AD5" s="5"/>
-      <c r="AE5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="AF5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="AM5" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE5" s="10"/>
+      <c r="AF5" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG5" s="10"/>
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="10"/>
+      <c r="AJ5" s="10"/>
+      <c r="AK5" s="10"/>
+      <c r="AL5" s="10"/>
+      <c r="AM5" s="10"/>
+      <c r="AN5" s="10"/>
+      <c r="AO5" s="10"/>
+      <c r="AP5" s="10"/>
       <c r="AQ5" s="6"/>
     </row>
-    <row r="6" spans="1:43">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="K6" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="10"/>
+      <c r="E6" s="10"/>
+      <c r="F6" s="10"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
       <c r="O6" s="6"/>
       <c r="P6" s="5"/>
-      <c r="Y6" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S6" s="10"/>
+      <c r="T6" s="10"/>
+      <c r="U6" s="10"/>
+      <c r="V6" s="10"/>
+      <c r="W6" s="10"/>
+      <c r="X6" s="10"/>
+      <c r="Y6" s="10"/>
+      <c r="Z6" s="10"/>
+      <c r="AA6" s="10"/>
+      <c r="AB6" s="10"/>
       <c r="AC6" s="6"/>
       <c r="AD6" s="5"/>
-      <c r="AN6" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE6" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF6" s="10"/>
+      <c r="AG6" s="10"/>
+      <c r="AH6" s="10"/>
+      <c r="AI6" s="10"/>
+      <c r="AJ6" s="10"/>
+      <c r="AK6" s="10"/>
+      <c r="AL6" s="10"/>
+      <c r="AM6" s="10"/>
+      <c r="AN6" s="10"/>
+      <c r="AO6" s="10"/>
+      <c r="AP6" s="10"/>
       <c r="AQ6" s="6"/>
     </row>
-    <row r="7" spans="1:43">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B7" s="5"/>
-      <c r="M7" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="10"/>
+      <c r="E7" s="10"/>
+      <c r="F7" s="10"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
       <c r="O7" s="6"/>
       <c r="P7" s="5"/>
+      <c r="Q7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="R7" s="10"/>
+      <c r="S7" s="10"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="10"/>
+      <c r="V7" s="10"/>
+      <c r="W7" s="10"/>
+      <c r="X7" s="10"/>
+      <c r="Y7" s="10"/>
+      <c r="Z7" s="10"/>
+      <c r="AA7" s="10"/>
+      <c r="AB7" s="10"/>
       <c r="AC7" s="6"/>
       <c r="AD7" s="5"/>
+      <c r="AE7" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF7" s="10"/>
+      <c r="AG7" s="10"/>
+      <c r="AH7" s="10"/>
+      <c r="AI7" s="10"/>
+      <c r="AJ7" s="10"/>
+      <c r="AK7" s="10"/>
+      <c r="AL7" s="10"/>
+      <c r="AM7" s="10"/>
+      <c r="AN7" s="10"/>
+      <c r="AO7" s="10"/>
+      <c r="AP7" s="10"/>
       <c r="AQ7" s="6"/>
     </row>
-    <row r="8" spans="1:43">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="5"/>
-      <c r="J8" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
       <c r="O8" s="6"/>
       <c r="P8" s="5"/>
-      <c r="Y8" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S8" s="10"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="10"/>
+      <c r="V8" s="10"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="10"/>
+      <c r="Y8" s="10"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="10"/>
+      <c r="AB8" s="10"/>
       <c r="AC8" s="6"/>
       <c r="AD8" s="5"/>
-      <c r="AF8" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE8" s="10"/>
+      <c r="AF8" s="10"/>
+      <c r="AG8" s="10"/>
+      <c r="AH8" s="10"/>
+      <c r="AI8" s="10"/>
+      <c r="AJ8" s="10"/>
+      <c r="AK8" s="10"/>
+      <c r="AL8" s="10"/>
+      <c r="AM8" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AN8" s="10"/>
+      <c r="AO8" s="10"/>
+      <c r="AP8" s="10"/>
       <c r="AQ8" s="6"/>
     </row>
-    <row r="9" spans="1:43">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B9" s="5"/>
-      <c r="D9" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
       <c r="O9" s="6"/>
       <c r="P9" s="5"/>
-      <c r="Z9" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
+      <c r="S9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="T9" s="10"/>
+      <c r="U9" s="10"/>
+      <c r="V9" s="10"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="10"/>
+      <c r="Y9" s="10"/>
+      <c r="Z9" s="10"/>
+      <c r="AA9" s="10"/>
+      <c r="AB9" s="10"/>
       <c r="AC9" s="6"/>
       <c r="AD9" s="5"/>
-      <c r="AM9" s="4" t="s">
-        <v>44</v>
-      </c>
+      <c r="AE9" s="10"/>
+      <c r="AF9" s="10"/>
+      <c r="AG9" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AH9" s="10"/>
+      <c r="AI9" s="10"/>
+      <c r="AJ9" s="10"/>
+      <c r="AK9" s="10"/>
+      <c r="AL9" s="10"/>
+      <c r="AM9" s="10"/>
+      <c r="AN9" s="10"/>
+      <c r="AO9" s="10"/>
+      <c r="AP9" s="10"/>
       <c r="AQ9" s="6"/>
     </row>
-    <row r="10" spans="1:43" ht="15.75" thickBot="1">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="M10" s="8"/>
-      <c r="N10" s="8"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="8"/>
-      <c r="S10" s="8"/>
-      <c r="T10" s="8"/>
-      <c r="U10" s="8"/>
-      <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
-      <c r="Y10" s="8"/>
-      <c r="Z10" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="AA10" s="8"/>
-      <c r="AB10" s="8"/>
-      <c r="AC10" s="9"/>
-      <c r="AD10" s="7"/>
-      <c r="AE10" s="8"/>
-      <c r="AF10" s="8"/>
-      <c r="AG10" s="8"/>
-      <c r="AH10" s="8"/>
-      <c r="AI10" s="8"/>
-      <c r="AJ10" s="8"/>
-      <c r="AK10" s="8"/>
-      <c r="AL10" s="8"/>
-      <c r="AM10" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="AN10" s="8"/>
-      <c r="AO10" s="8"/>
-      <c r="AP10" s="8"/>
-      <c r="AQ10" s="9"/>
+        <v>46</v>
+      </c>
+      <c r="B10" s="5"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="5"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+      <c r="S10" s="10"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="10"/>
+      <c r="V10" s="10"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="10"/>
+      <c r="Y10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AA10" s="10"/>
+      <c r="AB10" s="10"/>
+      <c r="AC10" s="6"/>
+      <c r="AD10" s="5"/>
+      <c r="AE10" s="10"/>
+      <c r="AF10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG10" s="10"/>
+      <c r="AH10" s="10"/>
+      <c r="AI10" s="10"/>
+      <c r="AJ10" s="10"/>
+      <c r="AK10" s="10"/>
+      <c r="AL10" s="10"/>
+      <c r="AM10" s="10"/>
+      <c r="AN10" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO10" s="10"/>
+      <c r="AP10" s="10"/>
+      <c r="AQ10" s="6"/>
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="5"/>
+      <c r="C11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="5"/>
+      <c r="Q11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="R11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="S11" s="10"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="10"/>
+      <c r="V11" s="10"/>
+      <c r="W11" s="10"/>
+      <c r="X11" s="10"/>
+      <c r="Y11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="Z11" s="10"/>
+      <c r="AA11" s="10"/>
+      <c r="AB11" s="10"/>
+      <c r="AC11" s="6"/>
+      <c r="AD11" s="5"/>
+      <c r="AE11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG11" s="10"/>
+      <c r="AH11" s="10"/>
+      <c r="AI11" s="10"/>
+      <c r="AJ11" s="10"/>
+      <c r="AK11" s="10"/>
+      <c r="AL11" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="AM11" s="10"/>
+      <c r="AN11" s="10"/>
+      <c r="AO11" s="10"/>
+      <c r="AP11" s="10"/>
+      <c r="AQ11" s="6"/>
+    </row>
+    <row r="12" spans="1:43" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="7"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="7"/>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+      <c r="Z12" s="8"/>
+      <c r="AA12" s="8"/>
+      <c r="AB12" s="8"/>
+      <c r="AC12" s="9"/>
+      <c r="AD12" s="7"/>
+      <c r="AE12" s="8"/>
+      <c r="AF12" s="8"/>
+      <c r="AG12" s="8"/>
+      <c r="AH12" s="8"/>
+      <c r="AI12" s="8"/>
+      <c r="AJ12" s="8"/>
+      <c r="AK12" s="8"/>
+      <c r="AL12" s="8"/>
+      <c r="AM12" s="8"/>
+      <c r="AN12" s="8"/>
+      <c r="AO12" s="8"/>
+      <c r="AP12" s="8"/>
+      <c r="AQ12" s="9"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:AQ10">
-    <sortCondition ref="A3:A10"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1293,22 +1663,46 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A53D224C-BBC6-4C47-A910-604FF4C700F0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB92840D-8E81-4B75-BB61-8EA2A722440C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0AF43DF-0D86-4FC0-883F-6115E8FD1AD4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0AF43DF-0D86-4FC0-883F-6115E8FD1AD4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
+    <ds:schemaRef ds:uri="b0d30a24-05e2-4154-8fed-e579ddd987b0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB92840D-8E81-4B75-BB61-8EA2A722440C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A53D224C-BBC6-4C47-A910-604FF4C700F0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Preassignments.xlsx: add Gibbs (3 AT preassignments)
Adds a new staff row for Gibbs with AT preassignments on Tue A 2,
Thu B 4, and Tue C 5. All other staff rows unchanged.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/upload files/Preassignments.xlsx
+++ b/upload files/Preassignments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5a8cad284f0e3288/Desktop/GitHub Repo/CrewOps360/upload files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/matthewgibbs/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{362294AE-22E4-8142-B845-4D38BA446C05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5F9D1377-4533-46B2-B828-AC49CADCC8B0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D47E277B-91CA-B14B-80BF-6B453ACD26E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1395" yWindow="945" windowWidth="22995" windowHeight="13260" xr2:uid="{011E8F27-AA14-4802-A81C-8523FD4162A1}"/>
+    <workbookView xWindow="1400" yWindow="940" windowWidth="23000" windowHeight="13260" xr2:uid="{011E8F27-AA14-4802-A81C-8523FD4162A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="56">
   <si>
     <t>STAFF NAME</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t>Laterion</t>
+  </si>
+  <si>
+    <t>Gibbs</t>
   </si>
 </sst>
 </file>
@@ -703,56 +706,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F22AD928-7495-4B5C-89C3-15EF76B28594}">
-  <dimension ref="A1:AQ12"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AQ13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.5" style="4" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="7.83203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.5" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="7" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="7.5" style="4" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="7.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="7.5" style="4" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="8" style="4" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="6.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="7.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="7.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="7.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8.140625" style="4" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="7.42578125" style="4" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="6.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="7.28515625" style="4" bestFit="1" customWidth="1"/>
-    <col min="44" max="16384" width="9.140625" style="4"/>
+    <col min="25" max="25" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="7.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="8.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="6.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="7.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="8.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="7.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.6640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="44" max="16384" width="9.1640625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -883,7 +886,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>52</v>
       </c>
@@ -903,7 +906,7 @@
       </c>
       <c r="AQ2" s="6"/>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>53</v>
       </c>
@@ -923,7 +926,7 @@
       </c>
       <c r="AQ3" s="6"/>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>51</v>
       </c>
@@ -944,7 +947,7 @@
       </c>
       <c r="AQ4" s="6"/>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>43</v>
       </c>
@@ -964,7 +967,7 @@
       </c>
       <c r="AQ5" s="6"/>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>50</v>
       </c>
@@ -984,7 +987,7 @@
       </c>
       <c r="AQ6" s="6"/>
     </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>54</v>
       </c>
@@ -1004,7 +1007,7 @@
       </c>
       <c r="AQ7" s="6"/>
     </row>
-    <row r="8" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>49</v>
       </c>
@@ -1027,7 +1030,7 @@
       <c r="AM8" s="10"/>
       <c r="AQ8" s="6"/>
     </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>45</v>
       </c>
@@ -1047,7 +1050,7 @@
       </c>
       <c r="AQ9" s="6"/>
     </row>
-    <row r="10" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>46</v>
       </c>
@@ -1076,92 +1079,112 @@
       </c>
       <c r="AQ10" s="6"/>
     </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B11" s="5"/>
-      <c r="C11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="J11" s="4" t="s">
+      <c r="K11" s="4" t="s">
         <v>44</v>
       </c>
       <c r="O11" s="6"/>
       <c r="P11" s="5"/>
-      <c r="Q11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="R11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y11" s="4" t="s">
+      <c r="AA11" s="4" t="s">
         <v>44</v>
       </c>
       <c r="AC11" s="6"/>
       <c r="AD11" s="5"/>
-      <c r="AE11" s="4" t="s">
-        <v>44</v>
-      </c>
       <c r="AF11" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="AL11" s="4" t="s">
         <v>44</v>
       </c>
       <c r="AQ11" s="6"/>
     </row>
-    <row r="12" spans="1:43" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O12" s="6"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="Y12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC12" s="6"/>
+      <c r="AD12" s="5"/>
+      <c r="AE12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AL12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="AQ12" s="6"/>
+    </row>
+    <row r="13" spans="1:43" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
-      <c r="N12" s="8"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="8"/>
-      <c r="S12" s="8"/>
-      <c r="T12" s="8"/>
-      <c r="U12" s="8"/>
-      <c r="V12" s="8"/>
-      <c r="W12" s="8"/>
-      <c r="X12" s="8"/>
-      <c r="Y12" s="8"/>
-      <c r="Z12" s="8"/>
-      <c r="AA12" s="8"/>
-      <c r="AB12" s="8"/>
-      <c r="AC12" s="9"/>
-      <c r="AD12" s="7"/>
-      <c r="AE12" s="8"/>
-      <c r="AF12" s="8"/>
-      <c r="AG12" s="8"/>
-      <c r="AH12" s="8"/>
-      <c r="AI12" s="8"/>
-      <c r="AJ12" s="8"/>
-      <c r="AK12" s="8"/>
-      <c r="AL12" s="8"/>
-      <c r="AM12" s="8"/>
-      <c r="AN12" s="8"/>
-      <c r="AO12" s="8"/>
-      <c r="AP12" s="8"/>
-      <c r="AQ12" s="9"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="7"/>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+      <c r="Z13" s="8"/>
+      <c r="AA13" s="8"/>
+      <c r="AB13" s="8"/>
+      <c r="AC13" s="9"/>
+      <c r="AD13" s="7"/>
+      <c r="AE13" s="8"/>
+      <c r="AF13" s="8"/>
+      <c r="AG13" s="8"/>
+      <c r="AH13" s="8"/>
+      <c r="AI13" s="8"/>
+      <c r="AJ13" s="8"/>
+      <c r="AK13" s="8"/>
+      <c r="AL13" s="8"/>
+      <c r="AM13" s="8"/>
+      <c r="AN13" s="8"/>
+      <c r="AO13" s="8"/>
+      <c r="AP13" s="8"/>
+      <c r="AQ13" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1169,11 +1192,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1360,20 +1384,17 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="3ae64878-e7bb-4c65-a932-4cdc61fbe63f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A53D224C-BBC6-4C47-A910-604FF4C700F0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB92840D-8E81-4B75-BB61-8EA2A722440C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1398,9 +1419,11 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB92840D-8E81-4B75-BB61-8EA2A722440C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A53D224C-BBC6-4C47-A910-604FF4C700F0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3ae64878-e7bb-4c65-a932-4cdc61fbe63f"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>